<commit_message>
Update nightly research results
</commit_message>
<xml_diff>
--- a/reports/latest_investor_report.xlsx
+++ b/reports/latest_investor_report.xlsx
@@ -629,7 +629,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-09-12 06:36</t>
+          <t>Son Güncelleme: 2026-09-13 06:51</t>
         </is>
       </c>
       <c r="B3" s="2" t="n"/>
@@ -960,25 +960,25 @@
         </is>
       </c>
       <c r="D20" s="7" t="n">
-        <v>0.1319207930213133</v>
+        <v>0.1319207930213132</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>13192.07930213133</v>
+        <v>13192.07930213132</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>0.0437413188564415</v>
+        <v>0.0437413188564412</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>577.0389471339888</v>
+        <v>577.0389471339845</v>
       </c>
       <c r="H20" s="8" t="n">
-        <v>234.1111810047456</v>
+        <v>234.1111810047455</v>
       </c>
       <c r="I20" s="8" t="n">
         <v>213.0850028991699</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>0.8748263771288307</v>
+        <v>0.8748263771288256</v>
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
@@ -1003,25 +1003,25 @@
         </is>
       </c>
       <c r="D21" s="7" t="n">
-        <v>0.09914425429287414</v>
+        <v>0.09914425429287406</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>9914.425429287414</v>
+        <v>9914.425429287407</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>0.0171674480247481</v>
+        <v>0.0171674480247476</v>
       </c>
       <c r="G21" s="8" t="n">
-        <v>170.2053832525326</v>
+        <v>170.2053832525275</v>
       </c>
       <c r="H21" s="8" t="n">
-        <v>96.42747717689483</v>
+        <v>96.42747717689477</v>
       </c>
       <c r="I21" s="8" t="n">
-        <v>87.26794819863983</v>
+        <v>87.2679481986398</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>0.2160730580000092</v>
+        <v>0.2160730580000031</v>
       </c>
       <c r="K21" s="9" t="inlineStr">
         <is>
@@ -1044,16 +1044,16 @@
         </is>
       </c>
       <c r="D22" s="7" t="n">
-        <v>0.09732031456006449</v>
+        <v>0.09732031456006451</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>9732.031456006449</v>
+        <v>9732.031456006451</v>
       </c>
       <c r="F22" s="7" t="n">
         <v>0.0695500946938858</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>676.8637093291238</v>
+        <v>676.8637093291239</v>
       </c>
       <c r="H22" s="8" t="n">
         <v>426.2157127355135</v>
@@ -1103,7 +1103,7 @@
         <v>36.23975304114958</v>
       </c>
       <c r="J23" s="6" t="n">
-        <v>0.594290083864031</v>
+        <v>0.5942900838640295</v>
       </c>
       <c r="K23" s="10" t="inlineStr">
         <is>
@@ -1126,25 +1126,25 @@
         </is>
       </c>
       <c r="D24" s="7" t="n">
-        <v>0.08114172203589044</v>
+        <v>0.08114172203589055</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>8114.172203589044</v>
+        <v>8114.172203589055</v>
       </c>
       <c r="F24" s="7" t="n">
-        <v>0.0233118283326481</v>
+        <v>0.0233118283326483</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>189.1561894716127</v>
+        <v>189.1561894716146</v>
       </c>
       <c r="H24" s="8" t="n">
-        <v>136.5097916537755</v>
+        <v>136.5097916537756</v>
       </c>
       <c r="I24" s="8" t="n">
         <v>126.7299942016601</v>
       </c>
       <c r="J24" s="6" t="n">
-        <v>0.4662365666529613</v>
+        <v>0.4662365666529656</v>
       </c>
       <c r="K24" s="9" t="inlineStr">
         <is>
@@ -1243,7 +1243,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-09-12 06:36</t>
+          <t>Son Güncelleme: 2026-09-13 06:51</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1443,7 +1443,7 @@
         <v>0.0371203025212296</v>
       </c>
       <c r="F8" s="16" t="n">
-        <v>0.0437413188564415</v>
+        <v>0.0437413188564412</v>
       </c>
       <c r="G8" s="16" t="n">
         <v>0.120622641333925</v>
@@ -1452,7 +1452,7 @@
         <v>232.6260870205518</v>
       </c>
       <c r="I8" s="15" t="n">
-        <v>234.1111810047456</v>
+        <v>234.1111810047455</v>
       </c>
       <c r="J8" s="15" t="n">
         <v>251.3556618710683</v>
@@ -1554,7 +1554,7 @@
         <v>24.97999954223633</v>
       </c>
       <c r="E10" s="19" t="n">
-        <v>-0.07844690697526251</v>
+        <v>-0.0784469069752626</v>
       </c>
       <c r="F10" s="19" t="n">
         <v>-0.0190929272018391</v>
@@ -1563,7 +1563,7 @@
         <v>0.09315584596891301</v>
       </c>
       <c r="H10" s="18" t="n">
-        <v>23.02039584190442</v>
+        <v>23.02039584190441</v>
       </c>
       <c r="I10" s="18" t="n">
         <v>24.50305822947444</v>
@@ -1572,7 +1572,7 @@
         <v>27.30703253189641</v>
       </c>
       <c r="K10" s="18" t="n">
-        <v>23.02039584190442</v>
+        <v>23.02039584190441</v>
       </c>
       <c r="L10" s="17" t="inlineStr">
         <is>
@@ -1608,28 +1608,28 @@
         </is>
       </c>
       <c r="D11" s="15" t="n">
-        <v>94.80000305175781</v>
+        <v>94.8000030517578</v>
       </c>
       <c r="E11" s="16" t="n">
-        <v>-0.0794520528549532</v>
+        <v>-0.0794520528549533</v>
       </c>
       <c r="F11" s="16" t="n">
-        <v>0.0171674480247481</v>
+        <v>0.0171674480247476</v>
       </c>
       <c r="G11" s="16" t="n">
         <v>0.0870869998031074</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>87.26794819863983</v>
+        <v>87.2679481986398</v>
       </c>
       <c r="I11" s="15" t="n">
-        <v>96.42747717689483</v>
+        <v>96.42747717689477</v>
       </c>
       <c r="J11" s="15" t="n">
         <v>103.0558508988608</v>
       </c>
       <c r="K11" s="15" t="n">
-        <v>87.26794819863983</v>
+        <v>87.2679481986398</v>
       </c>
       <c r="L11" s="14" t="inlineStr">
         <is>
@@ -1668,10 +1668,10 @@
         <v>44.06000137329102</v>
       </c>
       <c r="E12" s="22" t="n">
-        <v>-0.084296702806661</v>
+        <v>-0.08429670280666079</v>
       </c>
       <c r="F12" s="22" t="n">
-        <v>0.0004088702928312</v>
+        <v>0.0004088702928311</v>
       </c>
       <c r="G12" s="22" t="n">
         <v>0.1101031122376878</v>
@@ -1731,7 +1731,7 @@
         <v>-0.0036968005684216</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>0.1486665754350491</v>
+        <v>0.1486665754350493</v>
       </c>
       <c r="H13" s="18" t="n">
         <v>424.0458804389618</v>
@@ -1740,7 +1740,7 @@
         <v>428.4103757555787</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>493.9266274370711</v>
+        <v>493.9266274370712</v>
       </c>
       <c r="K13" s="18" t="n">
         <v>408.5</v>
@@ -1782,7 +1782,7 @@
         <v>72.09999847412109</v>
       </c>
       <c r="E14" s="19" t="n">
-        <v>-0.1073109919236646</v>
+        <v>-0.1073109919236645</v>
       </c>
       <c r="F14" s="19" t="n">
         <v>-0.0366894684105838</v>
@@ -1839,7 +1839,7 @@
         <v>38.97999954223633</v>
       </c>
       <c r="E15" s="16" t="n">
-        <v>-0.0702987822798095</v>
+        <v>-0.0702987822798096</v>
       </c>
       <c r="F15" s="16" t="n">
         <v>0.0417778692166073</v>
@@ -1956,19 +1956,19 @@
         <v>-0.0353227048870178</v>
       </c>
       <c r="F17" s="16" t="n">
-        <v>0.0233118283326481</v>
+        <v>0.0233118283326483</v>
       </c>
       <c r="G17" s="16" t="n">
-        <v>0.1081830165120092</v>
+        <v>0.108183016512009</v>
       </c>
       <c r="H17" s="15" t="n">
         <v>128.6879452801489</v>
       </c>
       <c r="I17" s="15" t="n">
-        <v>136.5097916537755</v>
+        <v>136.5097916537756</v>
       </c>
       <c r="J17" s="15" t="n">
-        <v>147.8316076388897</v>
+        <v>147.8316076388896</v>
       </c>
       <c r="K17" s="15" t="n">
         <v>126.7299942016601</v>
@@ -2040,7 +2040,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-09-12 06:36</t>
+          <t>Son Güncelleme: 2026-09-13 06:51</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2151,7 +2151,7 @@
         <v>0.0195327504943525</v>
       </c>
       <c r="K4" s="16" t="n">
-        <v>0.0437413188564415</v>
+        <v>0.0437413188564412</v>
       </c>
     </row>
     <row r="5">
@@ -2260,10 +2260,10 @@
         </is>
       </c>
       <c r="E7" s="16" t="n">
-        <v>0.0821918345097203</v>
+        <v>0.0821918345097201</v>
       </c>
       <c r="F7" s="16" t="n">
-        <v>0.0349345483727359</v>
+        <v>0.0349345483727356</v>
       </c>
       <c r="G7" s="16" t="n">
         <v>0.0065102745953808</v>
@@ -2277,10 +2277,10 @@
         </is>
       </c>
       <c r="J7" s="16" t="n">
-        <v>0.0175239369224565</v>
+        <v>0.0175239369224564</v>
       </c>
       <c r="K7" s="16" t="n">
-        <v>0.0171674480247481</v>
+        <v>0.0171674480247476</v>
       </c>
     </row>
     <row r="8">
@@ -2323,7 +2323,7 @@
         <v>0.0291195183035908</v>
       </c>
       <c r="K8" s="22" t="n">
-        <v>0.0004088702928312</v>
+        <v>0.0004088702928311</v>
       </c>
     </row>
     <row r="9">
@@ -2352,7 +2352,7 @@
         <v>0.1359779535346976</v>
       </c>
       <c r="G9" s="19" t="n">
-        <v>0.2201541438032379</v>
+        <v>0.2201541438032381</v>
       </c>
       <c r="H9" s="19" t="n">
         <v>0.0096886004836262</v>
@@ -2406,7 +2406,7 @@
         </is>
       </c>
       <c r="J10" s="19" t="n">
-        <v>0.0242987733054774</v>
+        <v>0.0242987733054775</v>
       </c>
       <c r="K10" s="19" t="n">
         <v>-0.0366894684105838</v>
@@ -2449,7 +2449,7 @@
         </is>
       </c>
       <c r="J11" s="16" t="n">
-        <v>0.0244714614971411</v>
+        <v>0.0244714614971412</v>
       </c>
       <c r="K11" s="16" t="n">
         <v>0.0417778692166073</v>
@@ -2538,7 +2538,7 @@
         <v>0.0171812701253963</v>
       </c>
       <c r="K13" s="16" t="n">
-        <v>0.0233118283326481</v>
+        <v>0.0233118283326483</v>
       </c>
     </row>
     <row r="14">
@@ -2739,7 +2739,7 @@
         <v>-0.0537261855796603</v>
       </c>
       <c r="G18" s="24" t="n">
-        <v>-0.244328041464684</v>
+        <v>-0.2443280414646841</v>
       </c>
       <c r="H18" s="24" t="n">
         <v>-0.0419382538842088</v>
@@ -2750,7 +2750,7 @@
         </is>
       </c>
       <c r="J18" s="24" t="n">
-        <v>0.018326546308491</v>
+        <v>0.0183265463084909</v>
       </c>
       <c r="K18" s="24" t="n">
         <v>0.0999999076690971</v>
@@ -2793,7 +2793,7 @@
         </is>
       </c>
       <c r="J19" s="24" t="n">
-        <v>0.0139213599674617</v>
+        <v>0.0139213599674618</v>
       </c>
       <c r="K19" s="24" t="n">
         <v>0.0999999076690971</v>
@@ -2836,7 +2836,7 @@
         </is>
       </c>
       <c r="J20" s="24" t="n">
-        <v>0.0188455307128114</v>
+        <v>0.0188455307128113</v>
       </c>
       <c r="K20" s="24" t="n">
         <v>0.0294396733991557</v>
@@ -2872,7 +2872,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-09-12 06:36</t>
+          <t>Son Güncelleme: 2026-09-13 06:51</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2991,7 +2991,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-09-12 06:36</t>
+          <t>Son Güncelleme: 2026-09-13 06:51</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -3242,7 +3242,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-09-12 06:36</t>
+          <t>Son Güncelleme: 2026-09-13 06:51</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -3367,7 +3367,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Son Güncelleme: 2026-09-12 06:36</t>
+          <t>Son Güncelleme: 2026-09-13 06:51</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -3444,7 +3444,7 @@
         <v>-1763.40361076151</v>
       </c>
       <c r="G4" s="25" t="n">
-        <v>12035505.24630628</v>
+        <v>12217153.95918872</v>
       </c>
       <c r="H4" s="26" t="n">
         <v>0.0503429940619526</v>
@@ -3474,7 +3474,7 @@
         <v>402757.4632715508</v>
       </c>
       <c r="G5" s="25" t="n">
-        <v>12035505.24630628</v>
+        <v>12217153.95918872</v>
       </c>
       <c r="H5" s="26" t="n">
         <v>0.0503429940619526</v>
@@ -3504,7 +3504,7 @@
         <v>-56270.17347722268</v>
       </c>
       <c r="G6" s="25" t="n">
-        <v>12035505.24630628</v>
+        <v>12217153.95918872</v>
       </c>
       <c r="H6" s="26" t="n">
         <v>0.0503429940619526</v>
@@ -3525,16 +3525,16 @@
         <v>96.5</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>94.80000305175781</v>
+        <v>94.8000030517578</v>
       </c>
       <c r="E7" s="26" t="n">
-        <v>-0.01761654868644758</v>
+        <v>-0.01761654868644769</v>
       </c>
       <c r="F7" s="25" t="n">
-        <v>-1546.988053709545</v>
+        <v>-1546.98805370956</v>
       </c>
       <c r="G7" s="25" t="n">
-        <v>12035505.24630628</v>
+        <v>12217153.95918872</v>
       </c>
       <c r="H7" s="26" t="n">
         <v>0.0503429940619526</v>
@@ -3564,7 +3564,7 @@
         <v>-2067.772894119626</v>
       </c>
       <c r="G8" s="25" t="n">
-        <v>12035505.24630628</v>
+        <v>12217153.95918872</v>
       </c>
       <c r="H8" s="26" t="n">
         <v>0.0503429940619526</v>
@@ -3594,7 +3594,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="25" t="n">
-        <v>12035505.24630628</v>
+        <v>12217153.95918872</v>
       </c>
       <c r="H9" s="26" t="n">
         <v>0.0503429940619526</v>

</xml_diff>